<commit_message>
Fetch Nifty50 from Trendlyne
</commit_message>
<xml_diff>
--- a/sectoraldata.xlsx
+++ b/sectoraldata.xlsx
@@ -2852,13 +2852,13 @@
         <v>0.0476</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0154</v>
+        <v>0.0188</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0257</v>
+        <v>0.0269</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.0574</v>
+        <v>0.059</v>
       </c>
       <c r="G2" s="4" t="n"/>
     </row>
@@ -2873,13 +2873,13 @@
         <v>0.0687</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.06900000000000001</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0522</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.008800000000000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-0.1496</v>
+        <v>-0.1419</v>
       </c>
       <c r="G3" s="4" t="n"/>
     </row>
@@ -3202,7 +3202,7 @@
         <v>0.277</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>-0.007705851854819756</v>
+        <v>-0.007705851854819867</v>
       </c>
     </row>
     <row r="18">
@@ -3341,7 +3341,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: supplied Trendlyne screenshot; pattern column omitted.</t>
+          <t>Source: Trendlyne quarterly seasonality data, index ID 1887; pattern column omitted.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -3420,10 +3420,10 @@
         <v>0.103</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0549</v>
+        <v>0.0557</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0441</v>
+        <v>0.0246</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1156</v>
@@ -3441,10 +3441,10 @@
         <v>0.2071</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0071</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.004099999999999999</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.07049999999999999</v>
@@ -3988,10 +3988,10 @@
         <v>0.0645</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0433</v>
+        <v>0.0463</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.0182</v>
+        <v>-0.0073</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.0457</v>
@@ -4009,10 +4009,10 @@
         <v>0.07150000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.1026</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.08779999999999999</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0161</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.2106</v>
@@ -4556,10 +4556,10 @@
         <v>0.0433</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.08529999999999999</v>
+        <v>0.0901</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0554</v>
+        <v>0.0539</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1791</v>
@@ -4576,11 +4576,11 @@
       <c r="C3" s="3" t="n">
         <v>0.124</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>-0.004699999999999999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+      <c r="D3" s="3" t="n">
+        <v>0.0193</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0235</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.1158</v>
@@ -5124,10 +5124,10 @@
         <v>0.0775</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0128</v>
+        <v>0.0134</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0389</v>
+        <v>0.0486</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.09470000000000001</v>
@@ -5145,10 +5145,10 @@
         <v>0.1446</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0537</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0506</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0033</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0861</v>
@@ -5692,10 +5692,10 @@
         <v>0.0558</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.08130000000000001</v>
+        <v>0.08310000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.1299</v>
+        <v>0.1241</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.2819</v>
@@ -5713,10 +5713,10 @@
         <v>0.0786</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0653</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0561</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0098</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0698</v>
@@ -6260,10 +6260,10 @@
         <v>0.0762</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0218</v>
+        <v>0.0217</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0243</v>
+        <v>0.0388</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.0868</v>
@@ -6281,10 +6281,10 @@
         <v>0.1567</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0441</v>
+        <v>-0.0442</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.07049999999999999</v>
@@ -6828,10 +6828,10 @@
         <v>0.1313</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.06370000000000001</v>
+        <v>0.0658</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.04480000000000001</v>
+        <v>0.0431</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1562</v>
@@ -6849,10 +6849,10 @@
         <v>0.2502</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0217</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0322</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0102</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.1079</v>
@@ -7224,7 +7224,7 @@
         <v>0.0776</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>0.1125775597988938</v>
+        <v>0.1125775597988936</v>
       </c>
     </row>
     <row r="20">
@@ -7396,10 +7396,10 @@
         <v>0.1279</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0545</v>
+        <v>0.0565</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.04849999999999999</v>
+        <v>0.0392</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1355</v>
@@ -7417,10 +7417,10 @@
         <v>0.2407</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0104</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0203</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0097</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.0759</v>
@@ -7780,10 +7780,10 @@
         <v>0.1338</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0607</v>
+        <v>0.06309999999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0387</v>
+        <v>0.0261</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1406</v>
@@ -7800,11 +7800,11 @@
       <c r="C3" s="3" t="n">
         <v>0.2402</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>-0.0074</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+      <c r="D3" s="3" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0118</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.0542</v>
@@ -7831,7 +7831,7 @@
         <v>-0.0601</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.2238791606795894</v>
+        <v>0.2238791606795896</v>
       </c>
     </row>
     <row r="5">
@@ -7854,7 +7854,7 @@
         <v>0.2643</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.2958857927907836</v>
+        <v>0.2958857927907839</v>
       </c>
     </row>
     <row r="6">
@@ -8049,10 +8049,10 @@
         <v>0.1161</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0533</v>
+        <v>0.0555</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0453</v>
+        <v>0.0399</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1628</v>
@@ -8070,10 +8070,10 @@
         <v>0.1743</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0429</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0322</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0111</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.024</v>
@@ -8617,10 +8617,10 @@
         <v>0.1013</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0429</v>
+        <v>0.0451</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.016</v>
+        <v>0.0146</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1106</v>
@@ -8638,10 +8638,10 @@
         <v>0.1869</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.03700000000000001</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0263</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.011</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.005500000000000001</v>
@@ -9185,10 +9185,10 @@
         <v>0.1141</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0538</v>
+        <v>0.0557</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0379</v>
+        <v>0.0355</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1535</v>
@@ -9206,10 +9206,10 @@
         <v>0.1737</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0496</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0399</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.029</v>
@@ -9569,10 +9569,10 @@
         <v>0.1155</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0537</v>
+        <v>0.0557</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.034</v>
+        <v>0.0288</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1459</v>
@@ -9590,10 +9590,10 @@
         <v>0.1721</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0496</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0398</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0102</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0284</v>
@@ -10137,10 +10137,10 @@
         <v>0.0788</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0409</v>
+        <v>0.0429</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0321</v>
+        <v>0.0201</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.0859</v>
@@ -10158,10 +10158,10 @@
         <v>0.1419</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0549</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0451</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0103</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.062</v>
@@ -10372,7 +10372,7 @@
         <v>0.5447</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.2490933745523152</v>
+        <v>0.249093374552315</v>
       </c>
     </row>
     <row r="13">
@@ -10441,7 +10441,7 @@
         <v>0.4791</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.1724145446523677</v>
+        <v>0.1724145446523675</v>
       </c>
     </row>
     <row r="16">
@@ -10705,10 +10705,10 @@
         <v>0.1666</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0176</v>
+        <v>0.0206</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0581</v>
+        <v>0.0667</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1669</v>
@@ -10726,10 +10726,10 @@
         <v>0.274</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0066</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0215</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0146</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0489</v>
@@ -11273,10 +11273,10 @@
         <v>0.0329</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0361</v>
+        <v>0.0398</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0245</v>
+        <v>0.0248</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1094</v>
@@ -11294,10 +11294,10 @@
         <v>0.07290000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0677</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0493</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0193</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0405</v>
@@ -11841,10 +11841,10 @@
         <v>0.046</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0053</v>
+        <v>0.007800000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0319</v>
+        <v>0.04019999999999999</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.08</v>
@@ -11862,10 +11862,10 @@
         <v>0.0225</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0504</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0377</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0132</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.1436</v>
@@ -12409,10 +12409,10 @@
         <v>0.0669</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0389</v>
+        <v>0.04219999999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0234</v>
+        <v>0.0283</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.2466</v>
@@ -12430,10 +12430,10 @@
         <v>-0.0295</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0862</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0699</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0174</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.0385</v>
@@ -12690,7 +12690,7 @@
         <v>-0.1703</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>-0.01511520635920549</v>
+        <v>-0.01511520635920538</v>
       </c>
     </row>
     <row r="15">
@@ -12977,10 +12977,10 @@
         <v>-0.0412</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0289</v>
+        <v>0.0244</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.08839999999999999</v>
+        <v>0.0718</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>-0.0356</v>
@@ -12998,10 +12998,10 @@
         <v>-0.0951</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.07629999999999999</v>
+        <v>0.0535</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.0217</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.2529</v>
@@ -13545,7 +13545,7 @@
         <v>0.0706</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0166</v>
+        <v>0.0193</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>0.0332</v>
@@ -13566,10 +13566,10 @@
         <v>0.09710000000000001</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.08380000000000001</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0701</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0147</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.1052</v>
@@ -13895,7 +13895,7 @@
         <v>0.2165</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>-0.1555174013343747</v>
+        <v>-0.1555174013343749</v>
       </c>
     </row>
     <row r="18">
@@ -14113,10 +14113,10 @@
         <v>0.0919</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.06150000000000001</v>
+        <v>0.06519999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.004699999999999999</v>
+        <v>-0.004500000000000001</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.09820000000000001</v>
@@ -14134,10 +14134,10 @@
         <v>0.1142</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0566</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0384</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0189</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.1161</v>
@@ -14371,7 +14371,7 @@
         <v>-0.0247</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0.1551979544552577</v>
+        <v>0.1551979544552575</v>
       </c>
     </row>
     <row r="14">
@@ -14681,10 +14681,10 @@
         <v>0.0711</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0102</v>
+        <v>0.0115</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.006999999999999999</v>
+        <v>0.0076</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1044</v>
@@ -14702,10 +14702,10 @@
         <v>0.1403</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.08439999999999999</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0781</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0068</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.0301</v>
@@ -14755,7 +14755,7 @@
         <v>0.05139999999999999</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.1720912291202243</v>
+        <v>0.1720912291202246</v>
       </c>
     </row>
     <row r="6">
@@ -14778,7 +14778,7 @@
         <v>0.2937</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.1848319741569016</v>
+        <v>0.1848319741569018</v>
       </c>
     </row>
     <row r="7">
@@ -14801,7 +14801,7 @@
         <v>0.1431</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.1267035071207632</v>
+        <v>0.1267035071207634</v>
       </c>
     </row>
     <row r="8">
@@ -15249,10 +15249,10 @@
         <v>0.0591</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0658</v>
+        <v>0.0663</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0233</v>
+        <v>0.023</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1411</v>
@@ -15270,10 +15270,10 @@
         <v>0.1365</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0027</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.0001</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0026</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.09939999999999999</v>
@@ -15817,10 +15817,10 @@
         <v>0.05230000000000001</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0759</v>
+        <v>0.07690000000000001</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0221</v>
+        <v>0.0245</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1483</v>
@@ -15838,10 +15838,10 @@
         <v>0.1392</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.0389</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>0.04389999999999999</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0048</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>0.1579</v>
@@ -16385,10 +16385,10 @@
         <v>0.1515</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.0593</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.0165</v>
+        <v>0.0032</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>0.1982</v>
@@ -16406,10 +16406,10 @@
         <v>0.114</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-0.0413</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+        <v>-0.006999999999999999</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-0.0346</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>-0.09949999999999999</v>
@@ -16620,7 +16620,7 @@
         <v>0.3137</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.1998010910808794</v>
+        <v>0.1998010910808796</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Refresh sector data 2026-10-07
</commit_message>
<xml_diff>
--- a/sectoraldata.xlsx
+++ b/sectoraldata.xlsx
@@ -33,6 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commodities" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oil and gas" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPSE" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_RefreshStatus" sheetId="27" state="hidden" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3341,7 +3342,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1887; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1887; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -3909,7 +3910,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1926; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1926; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -4477,7 +4478,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1901; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1901; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -5045,7 +5046,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1904; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1904; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -5613,7 +5614,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1898; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1898; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -6181,7 +6182,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1906; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1906; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -6749,7 +6750,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910338; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910338; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -7317,7 +7318,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910396; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910396; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -7701,7 +7702,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1896; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1896; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -7970,7 +7971,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910398; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910398; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G12" s="4" t="n"/>
@@ -8538,7 +8539,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1894; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1894; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -9106,7 +9107,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1888; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1888; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -9490,7 +9491,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1895; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1895; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G17" s="4" t="n"/>
@@ -10058,7 +10059,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910393; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910393; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -10626,7 +10627,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910414; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910414; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -11194,7 +11195,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1907; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1907; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -11762,7 +11763,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1908; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1908; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -12330,7 +12331,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910411; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910411; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -12898,7 +12899,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1910; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1910; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -12906,6 +12907,484 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Last successful refresh</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last refresh attempt</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Nifty50</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Next50</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Consumption</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pharma</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Alpha50</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FMCG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BankNifty</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PSUBanks</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PrivateBank</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SmallCap50</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SmallCap100</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SmallCap250</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Midcap50</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Midcap100</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Midcap150</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Nifty200 Momentum30</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Realty</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Commodities</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Oil and gas</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CPSE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -13466,7 +13945,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1902; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1902; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -14034,7 +14513,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1911; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1911; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -14602,7 +15081,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1909; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1909; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -15170,7 +15649,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1899; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1899; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -15738,7 +16217,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 910417; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 910417; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -16306,7 +16785,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1905; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1905; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>
@@ -16874,7 +17353,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Source: Trendlyne quarterly seasonality data, index ID 1897; pattern column omitted.</t>
+          <t>Source: Trendlyne index ID 1897; last refresh failed, showing previously saved data.</t>
         </is>
       </c>
       <c r="G25" s="4" t="n"/>

</xml_diff>

<commit_message>
Refresh sector data 2026-10-09
</commit_message>
<xml_diff>
--- a/sectoraldata.xlsx
+++ b/sectoraldata.xlsx
@@ -12949,7 +12949,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -13000,7 +13000,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -13034,7 +13034,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -13051,7 +13051,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -13102,7 +13102,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -13136,7 +13136,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -13153,7 +13153,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -13204,7 +13204,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -13221,7 +13221,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -13255,7 +13255,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -13306,7 +13306,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -13323,7 +13323,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -13357,7 +13357,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -13374,7 +13374,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">

</xml_diff>